<commit_message>
chore(data): pipeline OK [price-only] 2026-07-02 08:00
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1600"/>
+  <dimension ref="A1:B1601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16430,6 +16430,16 @@
         <v>1542</v>
       </c>
     </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B1601" t="n">
+        <v>1552.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-03 08:22
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1601"/>
+  <dimension ref="A1:B1602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16440,6 +16440,16 @@
         <v>1552.5</v>
       </c>
     </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B1602" t="n">
+        <v>1542.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-07 07:57
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1602"/>
+  <dimension ref="A1:B1604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16450,6 +16450,26 @@
         <v>1542.5</v>
       </c>
     </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B1603" t="n">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B1604" t="n">
+        <v>1530.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-08 08:06
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1604"/>
+  <dimension ref="A1:B1605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16470,6 +16470,16 @@
         <v>1530.5</v>
       </c>
     </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B1605" t="n">
+        <v>1517.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-09 08:00
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1605"/>
+  <dimension ref="A1:B1606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16480,6 +16480,16 @@
         <v>1517.2</v>
       </c>
     </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B1606" t="n">
+        <v>1507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-10 07:57
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1606"/>
+  <dimension ref="A1:B1607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16490,6 +16490,16 @@
         <v>1507</v>
       </c>
     </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B1607" t="n">
+        <v>1507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-13 08:57
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1607"/>
+  <dimension ref="A1:B1609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16500,6 +16500,26 @@
         <v>1507</v>
       </c>
     </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B1608" t="n">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B1609" t="n">
+        <v>1502</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-20 10:50
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1609"/>
+  <dimension ref="A1:B1613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16520,6 +16520,46 @@
         <v>1502</v>
       </c>
     </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B1610" t="n">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B1611" t="n">
+        <v>1488.5</v>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B1612" t="n">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B1613" t="n">
+        <v>1484.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-22 08:53
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1613"/>
+  <dimension ref="A1:B1615"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16560,6 +16560,26 @@
         <v>1484.4</v>
       </c>
     </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B1614" t="n">
+        <v>1482.5</v>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B1615" t="n">
+        <v>1481</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-24 08:04
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1615"/>
+  <dimension ref="A1:B1616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16580,6 +16580,16 @@
         <v>1481</v>
       </c>
     </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B1616" t="n">
+        <v>1476.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-27 08:06
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1616"/>
+  <dimension ref="A1:B1617"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16590,6 +16590,16 @@
         <v>1476.5</v>
       </c>
     </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B1617" t="n">
+        <v>1462.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-28 08:16
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1617"/>
+  <dimension ref="A1:B1618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16600,6 +16600,16 @@
         <v>1462.5</v>
       </c>
     </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B1618" t="n">
+        <v>1466</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-29 08:01
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1618"/>
+  <dimension ref="A1:B1619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16610,6 +16610,16 @@
         <v>1466</v>
       </c>
     </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B1619" t="n">
+        <v>1455.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-30 07:50
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1619"/>
+  <dimension ref="A1:B1620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16620,6 +16620,16 @@
         <v>1455.2</v>
       </c>
     </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1620" t="n">
+        <v>1446</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-07-31 08:02
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1620"/>
+  <dimension ref="A1:B1621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16630,6 +16630,16 @@
         <v>1446</v>
       </c>
     </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1621" t="n">
+        <v>1426.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-03 07:56
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1621"/>
+  <dimension ref="A1:B1622"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16640,6 +16640,16 @@
         <v>1426.2</v>
       </c>
     </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1622" t="n">
+        <v>1440</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-08-04 10:43
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1622"/>
+  <dimension ref="A1:B1624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16650,6 +16650,26 @@
         <v>1440</v>
       </c>
     </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B1623" t="n">
+        <v>1430.8</v>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B1624" t="n">
+        <v>1424.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-05 12:49
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1624"/>
+  <dimension ref="A1:B1625"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16670,6 +16670,16 @@
         <v>1424.4</v>
       </c>
     </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B1625" t="n">
+        <v>1423.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-07 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1625"/>
+  <dimension ref="A1:B1626"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16680,6 +16680,16 @@
         <v>1423.6</v>
       </c>
     </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B1626" t="n">
+        <v>1424.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-10 08:14
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1626"/>
+  <dimension ref="A1:B1627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16690,6 +16690,16 @@
         <v>1424.5</v>
       </c>
     </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B1627" t="n">
+        <v>1411</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-08-11 08:24
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1627"/>
+  <dimension ref="A1:B1628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16700,6 +16700,16 @@
         <v>1411</v>
       </c>
     </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B1628" t="n">
+        <v>1419.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-11 10:16
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1628"/>
+  <dimension ref="A1:B1629"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16710,6 +16710,16 @@
         <v>1419.5</v>
       </c>
     </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B1629" t="n">
+        <v>1413.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-13 08:05
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1629"/>
+  <dimension ref="A1:B1630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16720,6 +16720,16 @@
         <v>1413.4</v>
       </c>
     </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B1630" t="n">
+        <v>1419</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-14 08:11
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1630"/>
+  <dimension ref="A1:B1631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16730,6 +16730,16 @@
         <v>1419</v>
       </c>
     </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B1631" t="n">
+        <v>1420.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-18 08:01
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1631"/>
+  <dimension ref="A1:B1632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16740,6 +16740,16 @@
         <v>1420.2</v>
       </c>
     </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B1632" t="n">
+        <v>1417.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-19 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1632"/>
+  <dimension ref="A1:B1633"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16750,6 +16750,16 @@
         <v>1417.5</v>
       </c>
     </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B1633" t="n">
+        <v>1413.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-20 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1633"/>
+  <dimension ref="A1:B1634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16760,6 +16760,16 @@
         <v>1413.5</v>
       </c>
     </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B1634" t="n">
+        <v>1390</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-20 14:31
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1634"/>
+  <dimension ref="A1:B1635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16770,6 +16770,16 @@
         <v>1390</v>
       </c>
     </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B1635" t="n">
+        <v>1394.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-24 08:12
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1635"/>
+  <dimension ref="A1:B1636"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16780,6 +16780,16 @@
         <v>1394.3</v>
       </c>
     </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B1636" t="n">
+        <v>1387</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-24 08:59
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1636"/>
+  <dimension ref="A1:B1637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16790,6 +16790,16 @@
         <v>1387</v>
       </c>
     </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B1637" t="n">
+        <v>1385.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-25 08:28
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1637"/>
+  <dimension ref="A1:B1638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16800,6 +16800,16 @@
         <v>1385.5</v>
       </c>
     </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B1638" t="n">
+        <v>1383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-08-26 13:31
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1638"/>
+  <dimension ref="A1:B1639"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16810,6 +16810,16 @@
         <v>1383</v>
       </c>
     </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B1639" t="n">
+        <v>1384.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-08-28 08:06
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1639"/>
+  <dimension ref="A1:B1640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16820,6 +16820,16 @@
         <v>1384.8</v>
       </c>
     </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B1640" t="n">
+        <v>1382</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [full] 2026-08-31 08:49
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1640"/>
+  <dimension ref="A1:B1642"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16830,6 +16830,26 @@
         <v>1382</v>
       </c>
     </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B1641" t="n">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B1642" t="n">
+        <v>1380</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-02 08:03
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1642"/>
+  <dimension ref="A1:B1643"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16850,6 +16850,16 @@
         <v>1380</v>
       </c>
     </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B1643" t="n">
+        <v>1375.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-03 07:54
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1643"/>
+  <dimension ref="A1:B1644"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16860,6 +16860,16 @@
         <v>1375.5</v>
       </c>
     </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B1644" t="n">
+        <v>1360.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-08 08:07
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1644"/>
+  <dimension ref="A1:B1647"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16870,6 +16870,36 @@
         <v>1360.3</v>
       </c>
     </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B1645" t="n">
+        <v>1358.5</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B1646" t="n">
+        <v>1349.5</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B1647" t="n">
+        <v>1347</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): pipeline OK [price-only] 2026-09-10 09:19
</commit_message>
<xml_diff>
--- a/data/0_raw/exchange_rate_data.xlsx
+++ b/data/0_raw/exchange_rate_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1647"/>
+  <dimension ref="A1:B1650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16900,6 +16900,36 @@
         <v>1347</v>
       </c>
     </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B1648" t="n">
+        <v>1341.5</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B1649" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B1650" t="n">
+        <v>1338.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>